<commit_message>
Add GM Info tab, hide rookie OVR in Rosters, remove display of need weights
</commit_message>
<xml_diff>
--- a/Files/TestFiles/GMInfo.xlsx
+++ b/Files/TestFiles/GMInfo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Important Files/Madden 25/DraftTool/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40f61192ff96ff75/Documents/Git/MaddenDraftTool/Files/TestFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{81505719-928E-4932-9F80-664CB85D07C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B202C20B-3D7D-4A27-8DA0-8366A3EEC574}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{81505719-928E-4932-9F80-664CB85D07C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{391C4F84-B6C4-568F-A8A2-4F5F3B28632D}"/>
   <bookViews>
-    <workbookView xWindow="3810" yWindow="4485" windowWidth="13005" windowHeight="8700" xr2:uid="{D9E70525-0270-488C-BDD7-416A590B3624}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D9E70525-0270-488C-BDD7-416A590B3624}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -252,6 +252,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>